<commit_message>
three stage pipeline -(slot --> room --> teacher) completed
</commit_message>
<xml_diff>
--- a/backend/uploads/exam_data.xlsx
+++ b/backend/uploads/exam_data.xlsx
@@ -469,7 +469,11 @@
       <c r="D2" t="n">
         <v>25</v>
       </c>
-      <c r="E2" t="inlineStr"/>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -488,7 +492,11 @@
       <c r="D3" t="n">
         <v>20</v>
       </c>
-      <c r="E3" t="inlineStr"/>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -507,7 +515,11 @@
       <c r="D4" t="n">
         <v>18</v>
       </c>
-      <c r="E4" t="inlineStr"/>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -681,7 +693,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B21"/>
+  <dimension ref="A1:B210"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -699,7 +711,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Student1</t>
+          <t>S001</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -711,67 +723,67 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Student1</t>
+          <t>S001</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>C4</t>
+          <t>C3</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Student2</t>
+          <t>S002</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>C1</t>
+          <t>C2</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Student2</t>
+          <t>S002</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>C2</t>
+          <t>C1</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Student3</t>
+          <t>S002</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>C2</t>
+          <t>C3</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Student3</t>
+          <t>S003</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>C3</t>
+          <t>C1</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Student4</t>
+          <t>S003</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -783,156 +795,2424 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Student4</t>
+          <t>S004</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>C5</t>
+          <t>C1</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Student5</t>
+          <t>S004</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>C4</t>
+          <t>C10</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Student5</t>
+          <t>S004</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>C6</t>
+          <t>C3</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Student6</t>
+          <t>S005</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>C6</t>
+          <t>C2</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Student6</t>
+          <t>S005</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>C7</t>
+          <t>C3</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Student7</t>
+          <t>S006</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>C7</t>
+          <t>C2</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Student7</t>
+          <t>S006</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>C8</t>
+          <t>C3</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Student8</t>
+          <t>S007</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>C8</t>
+          <t>C2</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Student8</t>
+          <t>S007</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>C9</t>
+          <t>C10</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Student9</t>
+          <t>S007</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>C9</t>
+          <t>C3</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Student9</t>
+          <t>S008</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>C10</t>
+          <t>C2</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Student10</t>
+          <t>S008</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>C10</t>
+          <t>C3</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Student10</t>
+          <t>S009</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
+          <t>C3</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>S009</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>C2</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>S009</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
           <t>C1</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>S010</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>C3</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>S010</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>S011</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>C10</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>S011</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>S012</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>C3</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>S012</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>C10</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>S012</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>C2</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>S013</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>C10</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>S013</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>C3</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>S014</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>C10</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>S014</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>S015</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>C3</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>S015</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>C10</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>S015</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>S016</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>S016</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>C3</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>S017</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>C3</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>S017</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>S018</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>S018</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>C2</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>S019</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>C10</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>S019</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>C3</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>S019</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>C2</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>S020</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>C3</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>S020</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>C2</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>S021</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>C3</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>S021</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>C10</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>S022</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>C2</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>S023</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>C2</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>S023</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>C10</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>S024</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>C10</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>S024</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>S025</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>S025</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>C10</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>S026</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>C10</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>S026</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>C2</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>S026</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>S027</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>S028</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>C10</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>S028</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>C2</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>S029</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>S030</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>C10</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>S031</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>S032</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>S033</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>S034</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>S035</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>S036</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>S037</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>S038</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>S039</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>C2</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>S040</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>C2</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>S041</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>C2</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>S042</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>C2</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>S043</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>C2</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>S044</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>C2</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>S045</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>C10</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>S046</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>C10</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>S047</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>C6</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>S047</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>C5</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>S047</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>S048</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>S048</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>C5</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>S049</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>S049</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>C6</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>S050</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>C6</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>S050</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>S051</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>C6</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>S051</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>S051</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>C5</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>S052</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>C6</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>S052</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>C5</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>S052</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>S053</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>C6</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>S053</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>S054</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>C6</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>S054</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>C5</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>S054</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>S055</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>C5</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>S055</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>S055</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>C6</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>S056</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>C6</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>S056</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>C5</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>S057</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>C6</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>S057</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>S058</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>C6</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>S058</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>S058</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>C5</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>S059</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>S059</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>C6</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>S059</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>C5</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>S060</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>S060</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>C6</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>S060</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>C5</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>S061</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>S061</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>C6</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>S061</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>C5</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>S062</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>S062</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>C5</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>S063</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>C6</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>S063</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>S064</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>C6</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>S064</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>C5</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>S065</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>C5</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>S065</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>C6</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>S066</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>C6</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>S066</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>S067</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>C5</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>S067</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>C6</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>S067</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>S068</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>S068</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>C5</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>S069</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>C5</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>S069</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>S070</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>S071</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>S073</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>C5</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>S074</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>C5</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>S075</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>C5</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>S076</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>C5</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>S077</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>C5</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>S078</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>C5</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>S079</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>C5</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>S080</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>C8</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>S080</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>C9</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>S081</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>C7</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>S081</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>C9</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>S082</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>C8</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>S082</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>C9</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>S082</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>C7</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>S083</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>C9</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>S083</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>C7</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>S083</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>C8</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>S084</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>C8</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>S084</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>C9</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>S085</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>C7</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>S085</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>C9</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>S086</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>C9</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>S086</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>C8</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>S087</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>C8</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>S087</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>C7</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>S088</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>C8</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>S088</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>C7</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>S088</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>C9</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>S089</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>C9</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>S089</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>C7</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>S089</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>C8</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>S090</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>C7</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>S090</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>C9</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>S091</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>C8</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>S091</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>C9</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>S092</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>C7</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>S092</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>C8</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>S092</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>C9</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>S093</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>C8</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>S093</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>C7</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>S094</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>C8</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>S094</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>C9</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>S094</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>C7</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>S095</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>C9</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>S095</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>C8</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>S095</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>C7</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>S096</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>C8</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>S096</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>C7</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>S097</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>C9</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>S097</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>C7</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>S098</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>C7</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>S098</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>C9</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>S098</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>C8</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>S099</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>C7</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>S099</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>C9</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>S100</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>C7</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>S100</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>C9</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>S101</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>C8</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>S101</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>C7</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>S102</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>C9</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>S102</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>C7</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>S103</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>C8</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>S103</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>C9</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>S104</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>C7</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>S104</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>C8</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>S105</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>C7</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>S106</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>C8</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>S107</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>C8</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>S108</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>C8</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>S109</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>C8</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>S110</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>C8</t>
         </is>
       </c>
     </row>
@@ -969,7 +3249,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>40</v>
+        <v>15</v>
       </c>
     </row>
     <row r="3">
@@ -979,7 +3259,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>35</v>
+        <v>15</v>
       </c>
     </row>
     <row r="4">
@@ -989,7 +3269,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
     </row>
     <row r="5">
@@ -999,7 +3279,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
     </row>
     <row r="6">
@@ -1009,7 +3289,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>45</v>
+        <v>25</v>
       </c>
     </row>
     <row r="7">
@@ -1019,7 +3299,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>60</v>
+        <v>25</v>
       </c>
     </row>
   </sheetData>
@@ -1033,7 +3313,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:C19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1112,12 +3392,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Dr. Verma</t>
+          <t>Dr. Joshi</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Squad</t>
+          <t>Senior</t>
         </is>
       </c>
     </row>
@@ -1129,7 +3409,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Dr. Reddy</t>
+          <t>Dr. Verma</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -1146,7 +3426,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Dr. Iyer</t>
+          <t>Dr. Reddy</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -1163,12 +3443,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Dr. Patel</t>
+          <t>Dr. Iyer</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Junior</t>
+          <t>Squad</t>
         </is>
       </c>
     </row>
@@ -1180,12 +3460,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Dr. Gupta</t>
+          <t>Dr. Kulkarni</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Junior</t>
+          <t>Squad</t>
         </is>
       </c>
     </row>
@@ -1197,7 +3477,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Dr. Khan</t>
+          <t>Dr. Patel</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1214,7 +3494,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Dr. Das</t>
+          <t>Dr. Gupta</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1231,7 +3511,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Dr. Joshi</t>
+          <t>Dr. Khan</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1248,7 +3528,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Dr. Singh</t>
+          <t>Dr. Das</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1265,7 +3545,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Dr. Kulkarni</t>
+          <t>Dr. Singh</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1320,6 +3600,40 @@
         </is>
       </c>
       <c r="C17" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>T17</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Dr. Bhatt</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>T18</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Dr. Mishra</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
         <is>
           <t>Junior</t>
         </is>
@@ -1336,7 +3650,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B17"/>
+  <dimension ref="A1:B19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1383,7 +3697,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>1,3</t>
+          <t>3,4</t>
         </is>
       </c>
     </row>
@@ -1395,7 +3709,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>1,2</t>
+          <t>1,4</t>
         </is>
       </c>
     </row>
@@ -1407,7 +3721,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2,3</t>
+          <t>1,2</t>
         </is>
       </c>
     </row>
@@ -1419,7 +3733,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>1,3</t>
+          <t>2,3</t>
         </is>
       </c>
     </row>
@@ -1431,7 +3745,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3,4</t>
         </is>
       </c>
     </row>
@@ -1443,7 +3757,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>1,4</t>
         </is>
       </c>
     </row>
@@ -1479,7 +3793,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -1540,6 +3854,30 @@
       <c r="B17" t="inlineStr">
         <is>
           <t>3</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>T17</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>T18</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>4</t>
         </is>
       </c>
     </row>

</xml_diff>